<commit_message>
feat(item-search): owner-directed date-block coverage — TC-ISR-PRS-020 (prep-after-return validation: message + Search locked + Reset recovery, green) and TC-ISR-PRS-021 (12-month render cycle, expected-fail pinning the value-overspill defect: 7 of 12 months spill up to 30px on Prep, Return +23px, AM/PM outside the border); calendar helpers in the page object; MD/plan/inventory synced to 21 TCs; PRS run-all 22 passed; workbook rebuilt
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/encore/testcases/item-search/item-search-product-search.xlsx
+++ b/clients/encore/testcases/item-search/item-search-product-search.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="807" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="207">
   <si>
     <t>TC ID</t>
   </si>
@@ -572,22 +572,73 @@
     <t>The search panel returns with its values intact</t>
   </si>
   <si>
+    <t>TC-ISR-PRS-020</t>
+  </si>
+  <si>
+    <t>A Prep date after the Return date is rejected with a message</t>
+  </si>
+  <si>
+    <t>The Products page is open with default criteria (both dates on today)</t>
+  </si>
+  <si>
+    <t>1. Open the Prep Date Time calendar and pick a day in a later month</t>
+  </si>
+  <si>
+    <t>The field takes the future date</t>
+  </si>
+  <si>
+    <t>2. Read the panel</t>
+  </si>
+  <si>
+    <t>"Prep date cannot be after the return date." appears in red and the Search button is locked</t>
+  </si>
+  <si>
+    <t>3. Click Reset</t>
+  </si>
+  <si>
+    <t>Both dates return to today's defaults and the message clears</t>
+  </si>
+  <si>
+    <t>TC-ISR-PRS-021</t>
+  </si>
+  <si>
+    <t>A date value renders fully inside its box in every month</t>
+  </si>
+  <si>
+    <t>The Products page is open with default criteria</t>
+  </si>
+  <si>
+    <t>1. Pick the 22nd of each of the next twelve months on Prep Date Time, measuring the field after each pick</t>
+  </si>
+  <si>
+    <t>Every rendered value fits inside the field's box</t>
+  </si>
+  <si>
+    <t>2. Pick a wide date on Return Date Time and measure it</t>
+  </si>
+  <si>
+    <t>The value fits inside the box</t>
+  </si>
+  <si>
+    <t>Both fields return to defaults</t>
+  </si>
+  <si>
     <t>SUMMARY</t>
   </si>
   <si>
     <t>Item Search — Product Search</t>
   </si>
   <si>
-    <t>Automated: 19 / Pending: 0</t>
-  </si>
-  <si>
-    <t>Pass:19 Fail:0 Skipped:0 Blocked:0</t>
+    <t>Automated: 21 / Pending: 0</t>
+  </si>
+  <si>
+    <t>Pass:21 Fail:0 Skipped:0 Blocked:0</t>
   </si>
   <si>
     <t>Last Updated: 2026-09-01</t>
   </si>
   <si>
-    <t>d96ccb59875274442c18342f06a9aa9c3097f6ed8a4e1cb1fd5e32267acbe42c</t>
+    <t>49b6bbaa1b0534e99f83598cc30c0c62ecee0b835796d356c2fde35f8e610e29</t>
   </si>
 </sst>
 </file>
@@ -976,7 +1027,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M63"/>
+  <dimension ref="A1:M69"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -3493,45 +3544,291 @@
         <v>25</v>
       </c>
     </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>184</v>
+      </c>
+      <c r="B62" t="s">
+        <v>185</v>
+      </c>
+      <c r="C62" t="s">
+        <v>15</v>
+      </c>
+      <c r="D62" t="s">
+        <v>16</v>
+      </c>
+      <c r="E62" t="s">
+        <v>17</v>
+      </c>
+      <c r="F62" t="s">
+        <v>18</v>
+      </c>
+      <c r="G62" t="s">
+        <v>19</v>
+      </c>
+      <c r="H62" t="s">
+        <v>20</v>
+      </c>
+      <c r="I62" t="s">
+        <v>21</v>
+      </c>
+      <c r="J62" t="s">
+        <v>186</v>
+      </c>
+      <c r="K62" t="s">
+        <v>187</v>
+      </c>
+      <c r="L62" t="s">
+        <v>188</v>
+      </c>
+      <c r="M62" t="s">
+        <v>25</v>
+      </c>
+    </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A63" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F63" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G63" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="H63" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="I63" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="J63" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="K63" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L63" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M63" s="2" t="s">
-        <v>188</v>
+      <c r="A63" t="s">
+        <v>25</v>
+      </c>
+      <c r="B63" t="s">
+        <v>25</v>
+      </c>
+      <c r="C63" t="s">
+        <v>25</v>
+      </c>
+      <c r="D63" t="s">
+        <v>25</v>
+      </c>
+      <c r="E63" t="s">
+        <v>25</v>
+      </c>
+      <c r="F63" t="s">
+        <v>25</v>
+      </c>
+      <c r="G63" t="s">
+        <v>25</v>
+      </c>
+      <c r="H63" t="s">
+        <v>25</v>
+      </c>
+      <c r="I63" t="s">
+        <v>25</v>
+      </c>
+      <c r="J63" t="s">
+        <v>25</v>
+      </c>
+      <c r="K63" t="s">
+        <v>189</v>
+      </c>
+      <c r="L63" t="s">
+        <v>190</v>
+      </c>
+      <c r="M63" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>25</v>
+      </c>
+      <c r="B64" t="s">
+        <v>25</v>
+      </c>
+      <c r="C64" t="s">
+        <v>25</v>
+      </c>
+      <c r="D64" t="s">
+        <v>25</v>
+      </c>
+      <c r="E64" t="s">
+        <v>25</v>
+      </c>
+      <c r="F64" t="s">
+        <v>25</v>
+      </c>
+      <c r="G64" t="s">
+        <v>25</v>
+      </c>
+      <c r="H64" t="s">
+        <v>25</v>
+      </c>
+      <c r="I64" t="s">
+        <v>25</v>
+      </c>
+      <c r="J64" t="s">
+        <v>25</v>
+      </c>
+      <c r="K64" t="s">
+        <v>191</v>
+      </c>
+      <c r="L64" t="s">
+        <v>192</v>
+      </c>
+      <c r="M64" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>193</v>
+      </c>
+      <c r="B65" t="s">
+        <v>194</v>
+      </c>
+      <c r="C65" t="s">
+        <v>15</v>
+      </c>
+      <c r="D65" t="s">
+        <v>16</v>
+      </c>
+      <c r="E65" t="s">
+        <v>17</v>
+      </c>
+      <c r="F65" t="s">
+        <v>18</v>
+      </c>
+      <c r="G65" t="s">
+        <v>19</v>
+      </c>
+      <c r="H65" t="s">
+        <v>20</v>
+      </c>
+      <c r="I65" t="s">
+        <v>21</v>
+      </c>
+      <c r="J65" t="s">
+        <v>195</v>
+      </c>
+      <c r="K65" t="s">
+        <v>196</v>
+      </c>
+      <c r="L65" t="s">
+        <v>197</v>
+      </c>
+      <c r="M65" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>25</v>
+      </c>
+      <c r="B66" t="s">
+        <v>25</v>
+      </c>
+      <c r="C66" t="s">
+        <v>25</v>
+      </c>
+      <c r="D66" t="s">
+        <v>25</v>
+      </c>
+      <c r="E66" t="s">
+        <v>25</v>
+      </c>
+      <c r="F66" t="s">
+        <v>25</v>
+      </c>
+      <c r="G66" t="s">
+        <v>25</v>
+      </c>
+      <c r="H66" t="s">
+        <v>25</v>
+      </c>
+      <c r="I66" t="s">
+        <v>25</v>
+      </c>
+      <c r="J66" t="s">
+        <v>25</v>
+      </c>
+      <c r="K66" t="s">
+        <v>198</v>
+      </c>
+      <c r="L66" t="s">
+        <v>199</v>
+      </c>
+      <c r="M66" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>25</v>
+      </c>
+      <c r="B67" t="s">
+        <v>25</v>
+      </c>
+      <c r="C67" t="s">
+        <v>25</v>
+      </c>
+      <c r="D67" t="s">
+        <v>25</v>
+      </c>
+      <c r="E67" t="s">
+        <v>25</v>
+      </c>
+      <c r="F67" t="s">
+        <v>25</v>
+      </c>
+      <c r="G67" t="s">
+        <v>25</v>
+      </c>
+      <c r="H67" t="s">
+        <v>25</v>
+      </c>
+      <c r="I67" t="s">
+        <v>25</v>
+      </c>
+      <c r="J67" t="s">
+        <v>25</v>
+      </c>
+      <c r="K67" t="s">
+        <v>191</v>
+      </c>
+      <c r="L67" t="s">
+        <v>200</v>
+      </c>
+      <c r="M67" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A69" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="I69" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="J69" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K69" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L69" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M69" s="2" t="s">
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -3547,7 +3844,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>189</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>